<commit_message>
pathway pages draw every hit, not the top ten, and drop the chance line
</commit_message>
<xml_diff>
--- a/03_Pathway_Enrichment/02_Contrasts/c_data/02_contrasts.xlsx
+++ b/03_Pathway_Enrichment/02_Contrasts/c_data/02_contrasts.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7263" uniqueCount="2296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7257" uniqueCount="2293">
   <si>
     <t>sheet</t>
   </si>
@@ -6886,12 +6886,6 @@
     <t>3.3.1</t>
   </si>
   <si>
-    <t>tidyr</t>
-  </si>
-  <si>
-    <t>1.3.2</t>
-  </si>
-  <si>
     <t>tidyselect</t>
   </si>
   <si>
@@ -6899,9 +6893,6 @@
   </si>
   <si>
     <t>0.7.3</t>
-  </si>
-  <si>
-    <t>viridisLite</t>
   </si>
   <si>
     <t>withr</t>
@@ -46659,7 +46650,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -47096,7 +47087,7 @@
         <v>2288</v>
       </c>
       <c r="B40" t="s">
-        <v>2289</v>
+        <v>2224</v>
       </c>
       <c r="C40" t="s">
         <v>2211</v>
@@ -47104,10 +47095,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>2289</v>
+      </c>
+      <c r="B41" t="s">
         <v>2290</v>
-      </c>
-      <c r="B41" t="s">
-        <v>2224</v>
       </c>
       <c r="C41" t="s">
         <v>2211</v>
@@ -47121,28 +47112,6 @@
         <v>2292</v>
       </c>
       <c r="C42" t="s">
-        <v>2211</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" t="s">
-        <v>2293</v>
-      </c>
-      <c r="B43" t="s">
-        <v>2244</v>
-      </c>
-      <c r="C43" t="s">
-        <v>2211</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>2294</v>
-      </c>
-      <c r="B44" t="s">
-        <v>2295</v>
-      </c>
-      <c r="C44" t="s">
         <v>2211</v>
       </c>
     </row>

</xml_diff>

<commit_message>
pathway PDFs get the same heatmaps, one set of pages per collection
</commit_message>
<xml_diff>
--- a/03_Pathway_Enrichment/02_Contrasts/c_data/02_contrasts.xlsx
+++ b/03_Pathway_Enrichment/02_Contrasts/c_data/02_contrasts.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7257" uniqueCount="2293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7341" uniqueCount="2350">
   <si>
     <t>sheet</t>
   </si>
@@ -6640,6 +6640,24 @@
     <t>0dc36d2d3fb0960d7b9f4242bb0d9080</t>
   </si>
   <si>
+    <t>singscore</t>
+  </si>
+  <si>
+    <t>03_Pathway_Enrichment/01_Scores/c_data/singscore.rds</t>
+  </si>
+  <si>
+    <t>b1469538e9bdab96cd635a648fbe209e</t>
+  </si>
+  <si>
+    <t>phenotype</t>
+  </si>
+  <si>
+    <t>00_Input/phenotype.csv</t>
+  </si>
+  <si>
+    <t>5a1989db406daa0b70189a9f0df52cf3</t>
+  </si>
+  <si>
     <t>package</t>
   </si>
   <si>
@@ -6649,6 +6667,15 @@
     <t>source</t>
   </si>
   <si>
+    <t>BiocGenerics</t>
+  </si>
+  <si>
+    <t>0.58.0</t>
+  </si>
+  <si>
+    <t>Bioconductor 3.23 (R 4.6.0)</t>
+  </si>
+  <si>
     <t>BiocManager</t>
   </si>
   <si>
@@ -6664,7 +6691,22 @@
     <t>1.46.0</t>
   </si>
   <si>
-    <t>Bioconductor 3.23 (R 4.6.0)</t>
+    <t>bit</t>
+  </si>
+  <si>
+    <t>4.6.0</t>
+  </si>
+  <si>
+    <t>bit64</t>
+  </si>
+  <si>
+    <t>4.8.0</t>
+  </si>
+  <si>
+    <t>circlize</t>
+  </si>
+  <si>
+    <t>0.4.18</t>
   </si>
   <si>
     <t>cli</t>
@@ -6673,24 +6715,66 @@
     <t>3.6.6</t>
   </si>
   <si>
+    <t>clue</t>
+  </si>
+  <si>
+    <t>0.3-68</t>
+  </si>
+  <si>
+    <t>cluster</t>
+  </si>
+  <si>
+    <t>2.1.8.2</t>
+  </si>
+  <si>
     <t>codetools</t>
   </si>
   <si>
     <t>0.2-20</t>
   </si>
   <si>
+    <t>colorspace</t>
+  </si>
+  <si>
+    <t>2.1-2</t>
+  </si>
+  <si>
+    <t>ComplexHeatmap</t>
+  </si>
+  <si>
+    <t>2.28.0</t>
+  </si>
+  <si>
     <t>cowplot</t>
   </si>
   <si>
     <t>1.2.0</t>
   </si>
   <si>
+    <t>crayon</t>
+  </si>
+  <si>
+    <t>1.5.3</t>
+  </si>
+  <si>
     <t>data.table</t>
   </si>
   <si>
     <t>1.18.4</t>
   </si>
   <si>
+    <t>digest</t>
+  </si>
+  <si>
+    <t>0.6.39</t>
+  </si>
+  <si>
+    <t>doParallel</t>
+  </si>
+  <si>
+    <t>1.0.17</t>
+  </si>
+  <si>
     <t>dplyr</t>
   </si>
   <si>
@@ -6721,18 +6805,33 @@
     <t>1.38.0</t>
   </si>
   <si>
+    <t>foreach</t>
+  </si>
+  <si>
+    <t>1.5.2</t>
+  </si>
+  <si>
     <t>generics</t>
   </si>
   <si>
     <t>0.1.4</t>
   </si>
   <si>
+    <t>GetoptLong</t>
+  </si>
+  <si>
+    <t>1.1.1</t>
+  </si>
+  <si>
     <t>ggplot2</t>
   </si>
   <si>
     <t>4.0.3</t>
   </si>
   <si>
+    <t>GlobalOptions</t>
+  </si>
+  <si>
     <t>glue</t>
   </si>
   <si>
@@ -6751,6 +6850,24 @@
     <t>1.0.2</t>
   </si>
   <si>
+    <t>hms</t>
+  </si>
+  <si>
+    <t>1.1.4</t>
+  </si>
+  <si>
+    <t>IRanges</t>
+  </si>
+  <si>
+    <t>2.46.0</t>
+  </si>
+  <si>
+    <t>iterators</t>
+  </si>
+  <si>
+    <t>1.0.14</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -6787,6 +6904,12 @@
     <t>1.7-5</t>
   </si>
   <si>
+    <t>matrixStats</t>
+  </si>
+  <si>
+    <t>1.5.0</t>
+  </si>
+  <si>
     <t>pillar</t>
   </si>
   <si>
@@ -6799,6 +6922,12 @@
     <t>2.0.3</t>
   </si>
   <si>
+    <t>png</t>
+  </si>
+  <si>
+    <t>0.1-9</t>
+  </si>
+  <si>
     <t>purrr</t>
   </si>
   <si>
@@ -6823,12 +6952,24 @@
     <t>1.1.1-1.1</t>
   </si>
   <si>
+    <t>readr</t>
+  </si>
+  <si>
+    <t>2.2.0</t>
+  </si>
+  <si>
     <t>renv</t>
   </si>
   <si>
     <t>1.2.3</t>
   </si>
   <si>
+    <t>rjson</t>
+  </si>
+  <si>
+    <t>0.2.23</t>
+  </si>
+  <si>
     <t>rlang</t>
   </si>
   <si>
@@ -6844,6 +6985,12 @@
     <t>2.1.1</t>
   </si>
   <si>
+    <t>S4Vectors</t>
+  </si>
+  <si>
+    <t>0.50.0</t>
+  </si>
+  <si>
     <t>S7</t>
   </si>
   <si>
@@ -6862,6 +7009,12 @@
     <t>1.2.4</t>
   </si>
   <si>
+    <t>shape</t>
+  </si>
+  <si>
+    <t>1.4.6.1</t>
+  </si>
+  <si>
     <t>statmod</t>
   </si>
   <si>
@@ -6886,13 +7039,31 @@
     <t>3.3.1</t>
   </si>
   <si>
+    <t>tidyr</t>
+  </si>
+  <si>
+    <t>1.3.2</t>
+  </si>
+  <si>
     <t>tidyselect</t>
   </si>
   <si>
+    <t>tzdb</t>
+  </si>
+  <si>
+    <t>0.5.0</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
     <t>0.7.3</t>
+  </si>
+  <si>
+    <t>vroom</t>
+  </si>
+  <si>
+    <t>1.7.1</t>
   </si>
   <si>
     <t>withr</t>
@@ -46585,7 +46756,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -46641,6 +46812,28 @@
       </c>
       <c r="C5" t="s">
         <v>2205</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>2206</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2207</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>2209</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2210</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2211</v>
       </c>
     </row>
   </sheetData>
@@ -46650,469 +46843,755 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>2206</v>
+        <v>2212</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2207</v>
+        <v>2213</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2208</v>
+        <v>2214</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>2209</v>
+        <v>2215</v>
       </c>
       <c r="B2" t="s">
-        <v>2210</v>
+        <v>2216</v>
       </c>
       <c r="C2" t="s">
-        <v>2211</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>2212</v>
+        <v>2218</v>
       </c>
       <c r="B3" t="s">
-        <v>2213</v>
+        <v>2219</v>
       </c>
       <c r="C3" t="s">
-        <v>2214</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>2215</v>
+        <v>2221</v>
       </c>
       <c r="B4" t="s">
-        <v>2216</v>
+        <v>2222</v>
       </c>
       <c r="C4" t="s">
-        <v>2211</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>2217</v>
+        <v>2223</v>
       </c>
       <c r="B5" t="s">
-        <v>2218</v>
+        <v>2224</v>
       </c>
       <c r="C5" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>2219</v>
+        <v>2225</v>
       </c>
       <c r="B6" t="s">
+        <v>2226</v>
+      </c>
+      <c r="C6" t="s">
         <v>2220</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2211</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>2221</v>
+        <v>2227</v>
       </c>
       <c r="B7" t="s">
-        <v>2222</v>
+        <v>2228</v>
       </c>
       <c r="C7" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>2223</v>
+        <v>2229</v>
       </c>
       <c r="B8" t="s">
-        <v>2224</v>
+        <v>2230</v>
       </c>
       <c r="C8" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>2225</v>
+        <v>2231</v>
       </c>
       <c r="B9" t="s">
-        <v>2226</v>
+        <v>2232</v>
       </c>
       <c r="C9" t="s">
-        <v>2227</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>2228</v>
+        <v>2233</v>
       </c>
       <c r="B10" t="s">
-        <v>2229</v>
+        <v>2234</v>
       </c>
       <c r="C10" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>2230</v>
+        <v>2235</v>
       </c>
       <c r="B11" t="s">
-        <v>2231</v>
+        <v>2236</v>
       </c>
       <c r="C11" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>2237</v>
       </c>
       <c r="B12" t="s">
-        <v>2232</v>
+        <v>2238</v>
       </c>
       <c r="C12" t="s">
-        <v>2214</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>2233</v>
+        <v>2239</v>
       </c>
       <c r="B13" t="s">
-        <v>2234</v>
+        <v>2240</v>
       </c>
       <c r="C13" t="s">
-        <v>2211</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>2235</v>
+        <v>2241</v>
       </c>
       <c r="B14" t="s">
-        <v>2236</v>
+        <v>2242</v>
       </c>
       <c r="C14" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>2237</v>
+        <v>2243</v>
       </c>
       <c r="B15" t="s">
-        <v>2238</v>
+        <v>2244</v>
       </c>
       <c r="C15" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>2239</v>
+        <v>2245</v>
       </c>
       <c r="B16" t="s">
-        <v>2240</v>
+        <v>2246</v>
       </c>
       <c r="C16" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>2241</v>
+        <v>2247</v>
       </c>
       <c r="B17" t="s">
-        <v>2242</v>
+        <v>2248</v>
       </c>
       <c r="C17" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>2243</v>
+        <v>2249</v>
       </c>
       <c r="B18" t="s">
-        <v>2244</v>
+        <v>2250</v>
       </c>
       <c r="C18" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>2245</v>
+        <v>2251</v>
       </c>
       <c r="B19" t="s">
-        <v>2246</v>
+        <v>2252</v>
       </c>
       <c r="C19" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>2247</v>
+        <v>2253</v>
       </c>
       <c r="B20" t="s">
-        <v>2248</v>
+        <v>2254</v>
       </c>
       <c r="C20" t="s">
-        <v>2211</v>
+        <v>2255</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>2249</v>
+        <v>2256</v>
       </c>
       <c r="B21" t="s">
-        <v>2250</v>
+        <v>2257</v>
       </c>
       <c r="C21" t="s">
-        <v>2214</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>2251</v>
+        <v>2258</v>
       </c>
       <c r="B22" t="s">
-        <v>2252</v>
+        <v>2259</v>
       </c>
       <c r="C22" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>2253</v>
+        <v>42</v>
       </c>
       <c r="B23" t="s">
-        <v>2254</v>
+        <v>2260</v>
       </c>
       <c r="C23" t="s">
-        <v>2211</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>2255</v>
+        <v>2261</v>
       </c>
       <c r="B24" t="s">
-        <v>2256</v>
+        <v>2262</v>
       </c>
       <c r="C24" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>2257</v>
+        <v>2263</v>
       </c>
       <c r="B25" t="s">
-        <v>2258</v>
+        <v>2264</v>
       </c>
       <c r="C25" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>2259</v>
+        <v>2265</v>
       </c>
       <c r="B26" t="s">
-        <v>2260</v>
+        <v>2266</v>
       </c>
       <c r="C26" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>2261</v>
+        <v>2267</v>
       </c>
       <c r="B27" t="s">
-        <v>2262</v>
+        <v>2268</v>
       </c>
       <c r="C27" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>2263</v>
+        <v>2269</v>
       </c>
       <c r="B28" t="s">
         <v>2264</v>
       </c>
       <c r="C28" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="B29" t="s">
-        <v>2266</v>
+        <v>2271</v>
       </c>
       <c r="C29" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>2267</v>
+        <v>2272</v>
       </c>
       <c r="B30" t="s">
-        <v>2268</v>
+        <v>2273</v>
       </c>
       <c r="C30" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>2269</v>
+        <v>2274</v>
       </c>
       <c r="B31" t="s">
-        <v>2270</v>
+        <v>2275</v>
       </c>
       <c r="C31" t="s">
-        <v>2271</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>2272</v>
+        <v>2276</v>
       </c>
       <c r="B32" t="s">
-        <v>2273</v>
+        <v>2277</v>
       </c>
       <c r="C32" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>2274</v>
+        <v>2278</v>
       </c>
       <c r="B33" t="s">
-        <v>2275</v>
+        <v>2279</v>
       </c>
       <c r="C33" t="s">
-        <v>2211</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>2276</v>
+        <v>2280</v>
       </c>
       <c r="B34" t="s">
-        <v>2277</v>
+        <v>2281</v>
       </c>
       <c r="C34" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>2278</v>
+        <v>2282</v>
       </c>
       <c r="B35" t="s">
-        <v>2279</v>
+        <v>2283</v>
       </c>
       <c r="C35" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>2280</v>
+        <v>2284</v>
       </c>
       <c r="B36" t="s">
-        <v>2281</v>
+        <v>2285</v>
       </c>
       <c r="C36" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>2282</v>
+        <v>2286</v>
       </c>
       <c r="B37" t="s">
-        <v>2283</v>
+        <v>2287</v>
       </c>
       <c r="C37" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>2284</v>
+        <v>2288</v>
       </c>
       <c r="B38" t="s">
-        <v>2285</v>
+        <v>2289</v>
       </c>
       <c r="C38" t="s">
-        <v>2211</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>2286</v>
+        <v>2290</v>
       </c>
       <c r="B39" t="s">
-        <v>2287</v>
+        <v>2291</v>
       </c>
       <c r="C39" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>2288</v>
+        <v>2292</v>
       </c>
       <c r="B40" t="s">
-        <v>2224</v>
+        <v>2293</v>
       </c>
       <c r="C40" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>2289</v>
+        <v>2294</v>
       </c>
       <c r="B41" t="s">
-        <v>2290</v>
+        <v>2295</v>
       </c>
       <c r="C41" t="s">
-        <v>2211</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>2291</v>
+        <v>2296</v>
       </c>
       <c r="B42" t="s">
-        <v>2292</v>
+        <v>2297</v>
       </c>
       <c r="C42" t="s">
-        <v>2211</v>
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>2298</v>
+      </c>
+      <c r="B43" t="s">
+        <v>2299</v>
+      </c>
+      <c r="C43" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>2300</v>
+      </c>
+      <c r="B44" t="s">
+        <v>2301</v>
+      </c>
+      <c r="C44" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>2302</v>
+      </c>
+      <c r="B45" t="s">
+        <v>2303</v>
+      </c>
+      <c r="C45" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>2304</v>
+      </c>
+      <c r="B46" t="s">
+        <v>2305</v>
+      </c>
+      <c r="C46" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>2306</v>
+      </c>
+      <c r="B47" t="s">
+        <v>2307</v>
+      </c>
+      <c r="C47" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>2308</v>
+      </c>
+      <c r="B48" t="s">
+        <v>2309</v>
+      </c>
+      <c r="C48" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>2310</v>
+      </c>
+      <c r="B49" t="s">
+        <v>2311</v>
+      </c>
+      <c r="C49" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>2312</v>
+      </c>
+      <c r="B50" t="s">
+        <v>2313</v>
+      </c>
+      <c r="C50" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
+        <v>2314</v>
+      </c>
+      <c r="B51" t="s">
+        <v>2315</v>
+      </c>
+      <c r="C51" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>2316</v>
+      </c>
+      <c r="B52" t="s">
+        <v>2317</v>
+      </c>
+      <c r="C52" t="s">
+        <v>2318</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>2319</v>
+      </c>
+      <c r="B53" t="s">
+        <v>2320</v>
+      </c>
+      <c r="C53" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>2321</v>
+      </c>
+      <c r="B54" t="s">
+        <v>2322</v>
+      </c>
+      <c r="C54" t="s">
+        <v>2217</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>2323</v>
+      </c>
+      <c r="B55" t="s">
+        <v>2324</v>
+      </c>
+      <c r="C55" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>2325</v>
+      </c>
+      <c r="B56" t="s">
+        <v>2326</v>
+      </c>
+      <c r="C56" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>2327</v>
+      </c>
+      <c r="B57" t="s">
+        <v>2328</v>
+      </c>
+      <c r="C57" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>2329</v>
+      </c>
+      <c r="B58" t="s">
+        <v>2330</v>
+      </c>
+      <c r="C58" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>2331</v>
+      </c>
+      <c r="B59" t="s">
+        <v>2332</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>2333</v>
+      </c>
+      <c r="B60" t="s">
+        <v>2334</v>
+      </c>
+      <c r="C60" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>2335</v>
+      </c>
+      <c r="B61" t="s">
+        <v>2336</v>
+      </c>
+      <c r="C61" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>2337</v>
+      </c>
+      <c r="B62" t="s">
+        <v>2338</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>2339</v>
+      </c>
+      <c r="B63" t="s">
+        <v>2340</v>
+      </c>
+      <c r="C63" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>2341</v>
+      </c>
+      <c r="B64" t="s">
+        <v>2252</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>2342</v>
+      </c>
+      <c r="B65" t="s">
+        <v>2343</v>
+      </c>
+      <c r="C65" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>2344</v>
+      </c>
+      <c r="B66" t="s">
+        <v>2345</v>
+      </c>
+      <c r="C66" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>2346</v>
+      </c>
+      <c r="B67" t="s">
+        <v>2347</v>
+      </c>
+      <c r="C67" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>2348</v>
+      </c>
+      <c r="B68" t="s">
+        <v>2349</v>
+      </c>
+      <c r="C68" t="s">
+        <v>2220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
contrasts scripts join the shared block, and heat() keeps slice titles
</commit_message>
<xml_diff>
--- a/03_Pathway_Enrichment/02_Contrasts/c_data/02_contrasts.xlsx
+++ b/03_Pathway_Enrichment/02_Contrasts/c_data/02_contrasts.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7341" uniqueCount="2350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7344" uniqueCount="2352">
   <si>
     <t>sheet</t>
   </si>
@@ -7070,6 +7070,12 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>writexl</t>
+  </si>
+  <si>
+    <t>2.0.1</t>
   </si>
 </sst>
 </file>
@@ -46843,7 +46849,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -47594,6 +47600,17 @@
         <v>2220</v>
       </c>
     </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>2350</v>
+      </c>
+      <c r="B69" t="s">
+        <v>2351</v>
+      </c>
+      <c r="C69" t="s">
+        <v>2318</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>